<commit_message>
docs: agregar generalizacion Persona para Cliente y Domiciliario
</commit_message>
<xml_diff>
--- a/docs/diccionario_datos_domicilios .xlsx
+++ b/docs/diccionario_datos_domicilios .xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64668f439d6926d2/Documents/IdeaProjects/BlinkDelivery/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivanc\OneDrive\Escritorio\Talleres U\4to semestre\P3\BlinkDelivery\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6DC4EF4-BF53-4AC1-A2D4-2A817D44F92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814139D9-A426-4778-8836-F72CBE545CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Diccionario" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario!$A$1:$G$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="166">
   <si>
     <t>Tabla</t>
   </si>
@@ -43,9 +43,6 @@
     <t>cliente</t>
   </si>
   <si>
-    <t>Persona que usa la plataforma para pedir comida.</t>
-  </si>
-  <si>
     <t>Puede tener varias direcciones y hacer muchos pedidos (preguntas 1 y 4).</t>
   </si>
   <si>
@@ -97,12 +94,6 @@
     <t>domiciliario</t>
   </si>
   <si>
-    <t>Persona encargada de entregar los pedidos.</t>
-  </si>
-  <si>
-    <t>Se le asigna como máximo un pedido activo a la vez (pregunta 6).</t>
-  </si>
-  <si>
     <t>pedido</t>
   </si>
   <si>
@@ -160,24 +151,15 @@
     <t>PK</t>
   </si>
   <si>
-    <t>Identificador único del cliente.</t>
-  </si>
-  <si>
     <t>nombre</t>
   </si>
   <si>
     <t>VARCHAR(60)</t>
   </si>
   <si>
-    <t>Nombre del cliente, usado para identificarlo en la plataforma.</t>
-  </si>
-  <si>
     <t>apellido</t>
   </si>
   <si>
-    <t>Apellido del cliente.</t>
-  </si>
-  <si>
     <t>correo</t>
   </si>
   <si>
@@ -196,9 +178,6 @@
     <t>Sí</t>
   </si>
   <si>
-    <t>Número de contacto del cliente, útil para coordinar la entrega.</t>
-  </si>
-  <si>
     <t>contrasena_hash</t>
   </si>
   <si>
@@ -214,9 +193,6 @@
     <t>TIMESTAMP</t>
   </si>
   <si>
-    <t>Fecha en que el cliente creó su cuenta en la plataforma.</t>
-  </si>
-  <si>
     <t>id_direccion</t>
   </si>
   <si>
@@ -385,24 +361,9 @@
     <t>id_domiciliario</t>
   </si>
   <si>
-    <t>Identificador único del domiciliario.</t>
-  </si>
-  <si>
-    <t>Nombre del domiciliario.</t>
-  </si>
-  <si>
-    <t>Apellido del domiciliario.</t>
-  </si>
-  <si>
-    <t>Número de contacto, necesario para coordinar la entrega con cliente y restaurante.</t>
-  </si>
-  <si>
     <t>Disponibilidad actual del domiciliario (ej.: 'disponible', 'en entrega', 'inactivo').</t>
   </si>
   <si>
-    <t>Fecha de vinculación del domiciliario a la plataforma.</t>
-  </si>
-  <si>
     <t>id_pedido</t>
   </si>
   <si>
@@ -518,6 +479,54 @@
   </si>
   <si>
     <t>Fecha en que se registró la calificación.</t>
+  </si>
+  <si>
+    <t>persona.id_persona</t>
+  </si>
+  <si>
+    <t>Identificador del domiciliario. Es el mismo id_persona de la persona que tiene este rol; no se genera de forma independiente.</t>
+  </si>
+  <si>
+    <t>Fecha en que la persona se registró como domiciliario (inicio de ese rol).</t>
+  </si>
+  <si>
+    <t>Identificador del cliente. Es el mismo id_persona de la persona que tiene este rol; no se genera de forma independiente.</t>
+  </si>
+  <si>
+    <t>Fecha en que la persona se registró como cliente (inicio de ese rol).</t>
+  </si>
+  <si>
+    <t>persona</t>
+  </si>
+  <si>
+    <t>id_persona</t>
+  </si>
+  <si>
+    <t>Identificador único de la persona. Es la única identidad que se genera: cliente y domiciliario reutilizan este valor.</t>
+  </si>
+  <si>
+    <t>Nombre de la persona, compartido por todos sus roles.</t>
+  </si>
+  <si>
+    <t>Apellido de la persona.</t>
+  </si>
+  <si>
+    <t>Número de contacto. Opcional si la persona solo es cliente; obligatorio si la persona es domiciliario (RN26).</t>
+  </si>
+  <si>
+    <t>Rol (subtipo de persona) de quien usa la plataforma para pedir comida.</t>
+  </si>
+  <si>
+    <t>Rol (subtipo de persona) encargado de entregar los pedidos.</t>
+  </si>
+  <si>
+    <t>Se le asigna como máximo un pedido activo a la vez (pregunta 6); la persona debe tener teléfono (RN26).</t>
+  </si>
+  <si>
+    <t>Supertipo con los datos personales comunes (nombre, apellido, teléfono) de clientes y domiciliarios.</t>
+  </si>
+  <si>
+    <t>Evita duplicar datos personales. Generalización total y solapada: toda persona es cliente, domiciliario o ambos (RN25).</t>
   </si>
 </sst>
 </file>
@@ -624,7 +633,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -634,7 +643,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -908,7 +916,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -917,124 +925,135 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="39.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>155</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>164</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>161</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C10" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="39.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1045,7 +1064,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1058,743 +1077,749 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:7" s="3" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="D2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6" t="s">
-        <v>43</v>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>155</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>46</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>155</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="3" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
       <c r="G7" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>67</v>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="G11" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1" t="s">
-        <v>85</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>71</v>
+        <v>46</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>95</v>
+        <v>47</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="4" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" s="2" t="s">
+      <c r="G29" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2" t="s">
+    </row>
+    <row r="30" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" s="1" t="s">
+      <c r="C30" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1" t="s">
+    </row>
+    <row r="31" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" s="1" t="s">
         <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" s="4" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>113</v>
+        <v>79</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1"/>
+      <c r="G35" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="3" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>45</v>
-      </c>
       <c r="D37" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>52</v>
@@ -1803,31 +1828,33 @@
         <v>53</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A39" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1" t="s">
-        <v>122</v>
+      <c r="B39" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -1835,463 +1862,423 @@
         <v>21</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>58</v>
+      </c>
       <c r="G40" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>39</v>
+        <v>109</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>66</v>
+        <v>115</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>117</v>
+        <v>84</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>64</v>
+        <v>119</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F44" s="1" t="s">
-        <v>128</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
       <c r="G44" s="1" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>62</v>
+        <v>121</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>130</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
       <c r="G45" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>92</v>
+        <v>123</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B48" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F48" s="2"/>
+      <c r="G48" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="G49" s="1" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2" t="s">
-        <v>141</v>
+      <c r="A50" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1"/>
+      <c r="G51" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1"/>
+      <c r="G52" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B51" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F52" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="B53" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>148</v>
+        <v>111</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>113</v>
+        <v>56</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>129</v>
+      </c>
       <c r="G54" s="1" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F55" s="2"/>
-      <c r="G55" s="2" t="s">
-        <v>151</v>
+      <c r="A55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>124</v>
+        <v>74</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>152</v>
+        <v>57</v>
       </c>
       <c r="F56" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G56" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>39</v>
+        <v>143</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>66</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
       <c r="G57" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>82</v>
+        <v>146</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>103</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
       <c r="G58" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>157</v>
+        <v>53</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
       <c r="G59" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G61" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:G59" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: agregar vehiculo al domiciliario en esquema y diccionario
</commit_message>
<xml_diff>
--- a/docs/diccionario_datos_domicilios .xlsx
+++ b/docs/diccionario_datos_domicilios .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivanc\OneDrive\Escritorio\Talleres U\4to semestre\P3\BlinkDelivery\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{814139D9-A426-4778-8836-F72CBE545CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7810D1-7B86-4A42-A097-D6F2A5998BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Diccionario" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario!$A$1:$G$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario!$A$1:$G$60</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="168">
   <si>
     <t>Tabla</t>
   </si>
@@ -527,6 +527,12 @@
   </si>
   <si>
     <t>Evita duplicar datos personales. Generalización total y solapada: toda persona es cliente, domiciliario o ambos (RN25).</t>
+  </si>
+  <si>
+    <t>vehiculo</t>
+  </si>
+  <si>
+    <t>Tipo de vehículo con el que el domiciliario realiza las entregas: 'moto', 'bicicleta' o 'carro'.</t>
   </si>
 </sst>
 </file>
@@ -1064,7 +1070,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1798,23 +1804,23 @@
         <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="1" t="s">
+    <row r="37" spans="1:7" s="3" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" s="1" t="s">
+      <c r="B37" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D37" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1" t="s">
-        <v>110</v>
+      <c r="D37" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
@@ -1822,10 +1828,10 @@
         <v>20</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>38</v>
@@ -1833,59 +1839,55 @@
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
       <c r="G38" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B39" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E39" s="2" t="s">
+      <c r="D40" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2" t="s">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F40" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>56</v>
@@ -1897,10 +1899,10 @@
         <v>57</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
@@ -1908,75 +1910,79 @@
         <v>21</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>57</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>57</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>119</v>
+        <v>56</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
+      <c r="E44" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>117</v>
+      </c>
       <c r="G44" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>121</v>
+        <v>84</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>53</v>
+        <v>119</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>38</v>
@@ -1984,7 +1990,7 @@
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
       <c r="G45" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -1992,10 +1998,10 @@
         <v>21</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>105</v>
+        <v>53</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>38</v>
@@ -2003,70 +2009,66 @@
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B48" s="2" t="s">
+      <c r="B49" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="C49" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D48" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E48" s="2" t="s">
+      <c r="D49" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E49" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2" t="s">
+      <c r="F49" s="2"/>
+      <c r="G49" s="2" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="F49" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="G49" s="1" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -2074,7 +2076,7 @@
         <v>24</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>56</v>
@@ -2086,10 +2088,10 @@
         <v>57</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -2097,7 +2099,7 @@
         <v>24</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>56</v>
@@ -2105,21 +2107,25 @@
       <c r="D51" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
+      <c r="E51" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="G51" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>105</v>
+        <v>56</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>38</v>
@@ -2127,59 +2133,55 @@
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
       <c r="G52" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="2" t="s">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B54" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D53" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E53" s="2" t="s">
+      <c r="D54" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E54" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2" t="s">
+      <c r="F54" s="2"/>
+      <c r="G54" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>56</v>
@@ -2188,21 +2190,21 @@
         <v>38</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>57</v>
+        <v>139</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>58</v>
+        <v>129</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>56</v>
@@ -2214,29 +2216,33 @@
         <v>57</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>95</v>
+        <v>58</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>143</v>
+        <v>74</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>144</v>
+        <v>56</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
+      <c r="E57" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="G57" s="1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
@@ -2244,18 +2250,18 @@
         <v>27</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>79</v>
+        <v>144</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
       <c r="G58" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
@@ -2263,22 +2269,41 @@
         <v>27</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="E59" s="1"/>
       <c r="F59" s="1"/>
       <c r="G59" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1" t="s">
         <v>149</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G59" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:G60" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>